<commit_message>
Atualiza planilhas e imagens dos displays aramados
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO DISPLAY ARAMADO G.xlsx
+++ b/planilhas/LISTA DE PROCESSO DISPLAY ARAMADO G.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\PROJETOS EM ANDAMENTO\PAINEL DE CONTROLE MTECH\PROGRAMAS\PROJETOS - PAINEL PRODUÇÃO IA\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CE11555-9E02-41B0-B381-6BCEA103DF77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0289A0-E155-41E2-BFEF-016AB3DF8ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="81">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -231,6 +231,54 @@
   </si>
   <si>
     <t>Apoio Rodizio</t>
+  </si>
+  <si>
+    <t>0,75 Nest 1 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 2 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 3 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 4 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 5 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 6 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 7 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 8 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 9 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 10 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 11 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 12 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 13 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 14 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 15 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 16 AJUSTADA</t>
   </si>
 </sst>
 </file>
@@ -552,7 +600,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" bestFit="1" customWidth="1"/>
@@ -1650,6 +1698,326 @@
         <v>1198</v>
       </c>
     </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>19</v>
+      </c>
+      <c r="B54" t="s">
+        <v>20</v>
+      </c>
+      <c r="C54" t="s">
+        <v>13</v>
+      </c>
+      <c r="D54" t="s">
+        <v>65</v>
+      </c>
+      <c r="E54">
+        <v>3.6727879999999997E-2</v>
+      </c>
+      <c r="F54">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>19</v>
+      </c>
+      <c r="B55" t="s">
+        <v>20</v>
+      </c>
+      <c r="C55" t="s">
+        <v>13</v>
+      </c>
+      <c r="D55" t="s">
+        <v>66</v>
+      </c>
+      <c r="E55">
+        <v>8.3472500000000003E-4</v>
+      </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>19</v>
+      </c>
+      <c r="B56" t="s">
+        <v>20</v>
+      </c>
+      <c r="C56" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56" t="s">
+        <v>67</v>
+      </c>
+      <c r="E56">
+        <v>8.4307178999999996E-2</v>
+      </c>
+      <c r="F56">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>19</v>
+      </c>
+      <c r="B57" t="s">
+        <v>20</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57" t="s">
+        <v>68</v>
+      </c>
+      <c r="E57">
+        <v>2.3372286999999999E-2</v>
+      </c>
+      <c r="F57">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>19</v>
+      </c>
+      <c r="B58" t="s">
+        <v>20</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58" t="s">
+        <v>69</v>
+      </c>
+      <c r="E58">
+        <v>0.105175292</v>
+      </c>
+      <c r="F58">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>19</v>
+      </c>
+      <c r="B59" t="s">
+        <v>20</v>
+      </c>
+      <c r="C59" t="s">
+        <v>13</v>
+      </c>
+      <c r="D59" t="s">
+        <v>70</v>
+      </c>
+      <c r="E59">
+        <v>1.6694489999999999E-3</v>
+      </c>
+      <c r="F59">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>19</v>
+      </c>
+      <c r="B60" t="s">
+        <v>20</v>
+      </c>
+      <c r="C60" t="s">
+        <v>13</v>
+      </c>
+      <c r="D60" t="s">
+        <v>71</v>
+      </c>
+      <c r="E60">
+        <v>7.5125210000000003E-3</v>
+      </c>
+      <c r="F60">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>19</v>
+      </c>
+      <c r="B61" t="s">
+        <v>20</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61" t="s">
+        <v>72</v>
+      </c>
+      <c r="E61">
+        <v>8.3472500000000003E-4</v>
+      </c>
+      <c r="F61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>19</v>
+      </c>
+      <c r="B62" t="s">
+        <v>20</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62" t="s">
+        <v>73</v>
+      </c>
+      <c r="E62">
+        <v>8.3472500000000003E-4</v>
+      </c>
+      <c r="F62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>19</v>
+      </c>
+      <c r="B63" t="s">
+        <v>20</v>
+      </c>
+      <c r="C63" t="s">
+        <v>13</v>
+      </c>
+      <c r="D63" t="s">
+        <v>74</v>
+      </c>
+      <c r="E63">
+        <v>1.6694489999999999E-3</v>
+      </c>
+      <c r="F63">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>19</v>
+      </c>
+      <c r="B64" t="s">
+        <v>20</v>
+      </c>
+      <c r="C64" t="s">
+        <v>13</v>
+      </c>
+      <c r="D64" t="s">
+        <v>75</v>
+      </c>
+      <c r="E64">
+        <v>1.0016694E-2</v>
+      </c>
+      <c r="F64">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>19</v>
+      </c>
+      <c r="B65" t="s">
+        <v>20</v>
+      </c>
+      <c r="C65" t="s">
+        <v>13</v>
+      </c>
+      <c r="D65" t="s">
+        <v>76</v>
+      </c>
+      <c r="E65">
+        <v>1.6694489999999999E-3</v>
+      </c>
+      <c r="F65">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>19</v>
+      </c>
+      <c r="B66" t="s">
+        <v>20</v>
+      </c>
+      <c r="C66" t="s">
+        <v>13</v>
+      </c>
+      <c r="D66" t="s">
+        <v>77</v>
+      </c>
+      <c r="E66">
+        <v>5.0083469999999998E-3</v>
+      </c>
+      <c r="F66">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>19</v>
+      </c>
+      <c r="B67" t="s">
+        <v>20</v>
+      </c>
+      <c r="C67" t="s">
+        <v>13</v>
+      </c>
+      <c r="D67" t="s">
+        <v>78</v>
+      </c>
+      <c r="E67">
+        <v>2.1702837999999999E-2</v>
+      </c>
+      <c r="F67">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>19</v>
+      </c>
+      <c r="B68" t="s">
+        <v>20</v>
+      </c>
+      <c r="C68" t="s">
+        <v>13</v>
+      </c>
+      <c r="D68" t="s">
+        <v>79</v>
+      </c>
+      <c r="E68">
+        <v>3.0050082999999998E-2</v>
+      </c>
+      <c r="F68">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>19</v>
+      </c>
+      <c r="B69" t="s">
+        <v>20</v>
+      </c>
+      <c r="C69" t="s">
+        <v>13</v>
+      </c>
+      <c r="D69" t="s">
+        <v>80</v>
+      </c>
+      <c r="E69">
+        <v>8.3472500000000003E-4</v>
+      </c>
+      <c r="F69">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>